<commit_message>
corregido casos normales con abonos
</commit_message>
<xml_diff>
--- a/Excel/Libro de excel - Casos de prueba - Luisa Fernanda Espinal y Jose Manuel Jaramillo    (1) (1).xlsx
+++ b/Excel/Libro de excel - Casos de prueba - Luisa Fernanda Espinal y Jose Manuel Jaramillo    (1) (1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b12s308\Desktop\CalculadoraAhorroProgramado\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\b12s308\Desktop\cdl\CalculadoraAhorroProgramado\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B6883E9-65FD-428E-8E35-D296CD46FC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8640F061-D86B-4193-95CC-20BF57B568FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -739,8 +739,8 @@
         <v>0</v>
       </c>
       <c r="G4" s="15">
-        <f t="shared" ref="G4:G6" si="1">IF(OR(B4&lt;=0, C4&lt;=0), "Error", PMT(E4, C4, 0, -(B4-D4), 0))</f>
-        <v>179925.79819452611</v>
+        <f>IF(OR(B4&lt;=0,C4&lt;=0),"Error",(B4 - D4*(1+E4)^(C4-F4)) / (((1+E4)^C4-1)/E4))</f>
+        <v>179925.79819452376</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -754,18 +754,18 @@
         <v>12</v>
       </c>
       <c r="D5" s="12">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="E5" s="13">
         <f t="shared" si="0"/>
         <v>7.4999999999999997E-3</v>
       </c>
       <c r="F5" s="14">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G5" s="15">
-        <f t="shared" si="1"/>
-        <v>719563.29092929291</v>
+        <f t="shared" ref="G5:G6" si="1">IF(OR(B5&lt;=0,C5&lt;=0),"Error",(B5 - D5*(1+E5)^(C5-F5)) / (((1+E5)^C5-1)/E5))</f>
+        <v>635945.86024963693</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -790,7 +790,7 @@
       </c>
       <c r="G6" s="15">
         <f t="shared" si="1"/>
-        <v>4130954.5521899164</v>
+        <v>4130954.5521898647</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -845,7 +845,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="15">
-        <f t="shared" ref="G9:G11" si="2">(B9-D9)/C9</f>
+        <f t="shared" ref="G9" si="2">(B9-D9)/C9</f>
         <v>0</v>
       </c>
     </row>
@@ -869,7 +869,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="15">
-        <f t="shared" si="2"/>
+        <f>(B10-D10)/C10</f>
         <v>90000</v>
       </c>
     </row>
@@ -893,7 +893,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="15">
-        <f t="shared" si="2"/>
+        <f>(B11-D11)/C11</f>
         <v>0</v>
       </c>
     </row>
@@ -2031,6 +2031,6 @@
     <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>